<commit_message>
week2: local pipeline run outputs
</commit_message>
<xml_diff>
--- a/week2/data/sales_report_xw.xlsx
+++ b/week2/data/sales_report_xw.xlsx
@@ -162,9 +162,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>

</xml_diff>